<commit_message>
Stage 8 review fixes: E-013
</commit_message>
<xml_diff>
--- a/output/archive/WestravelleData/Stability/JO14/WA-2026-047/Results/Interim/JO14_FIRST_PULL_REVIEW_DRAFT_Rev01.xlsx
+++ b/output/archive/WestravelleData/Stability/JO14/WA-2026-047/Results/Interim/JO14_FIRST_PULL_REVIEW_DRAFT_Rev01.xlsx
@@ -162,18 +162,12 @@
 <file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
-    <author>Saira Mahmood</author>
     <author>Alice Penrose</author>
   </authors>
   <commentList>
-    <comment ref="A6" authorId="0" shapeId="0">
+    <comment ref="C13" authorId="0" shapeId="0">
       <text>
-        <t>Leon, can you confirm the chamber pull dates for the 3 and 6 month pulls? The tracker and the chamber log need to match before we send.</t>
-      </text>
-    </comment>
-    <comment ref="C12" authorId="1" shapeId="0">
-      <text>
-        <t>Sign-off column is blank for 3 and 6 months. Don't mark as reviewed until the chromatograms are checked.</t>
+        <t>First chamber-pull review remains open. Reconcile the timepoint entries with the chamber log and review chromatograms before completing sign-off. Later pulls remain pending.</t>
       </text>
     </comment>
   </commentList>
@@ -186,7 +180,7 @@
     <author>Saira Mahmood</author>
   </authors>
   <commentList>
-    <comment ref="F9" authorId="0" shapeId="0">
+    <comment ref="F15" authorId="0" shapeId="0">
       <text>
         <t>Total impurities at 40 °C, 3 months is above the 25 and 30 °C results at the same pull. Check the integration on the RRT 0.86 peak before we quote it externally.</t>
       </text>
@@ -201,9 +195,9 @@
     <author>Saira Mahmood</author>
   </authors>
   <commentList>
-    <comment ref="B7" authorId="0" shapeId="0">
+    <comment ref="B5" authorId="0" shapeId="0">
       <text>
-        <t>Linearity result is within criteria. Still need the signed range report from the QC system before this goes in the final package.</t>
+        <t>Linearity meets the acceptance criterion shown. Qualification is complete; attach the signed qualification record to the final package.</t>
       </text>
     </comment>
   </commentList>
@@ -664,14 +658,10 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Reported</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>Leon Wu</t>
-        </is>
-      </c>
+          <t>Results entered; review pending</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -684,14 +674,10 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Reported</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Leon Wu</t>
-        </is>
-      </c>
+          <t>Results entered; review pending</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -704,7 +690,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Reported, in review</t>
+          <t>Results entered; review pending</t>
         </is>
       </c>
       <c r="D12" s="2" t="n"/>
@@ -720,7 +706,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Reported, in review</t>
+          <t>Results entered; review pending</t>
         </is>
       </c>
       <c r="D13" s="2" t="n"/>

</xml_diff>